<commit_message>
Update soccer trades 2026-07-29 02:01:33 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,110 +643,222 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-29 20:01:43 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,110 +755,222 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-29 21:01:35 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,87 +546,87 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>36.47</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.2737</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19532655</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.5938</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19532532</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,110 +867,222 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 00:02:13 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,102 +531,94 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
+          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>36.47</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.2737</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19532655</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785356693</t>
+          <t>1785369486</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>133.223744</t>
+          <t>41.166667</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,87 +650,87 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>36.47</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.2737</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19532655</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.5938</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19532532</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,12 +762,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +777,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -795,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,7 +889,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -907,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,110 +971,222 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 14:02:27 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
+          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>47.67</t>
+          <t>178.29</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,32 +561,32 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785418294</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>138.676364</t>
+          <t>445.725</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +643,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
+          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>28.2797</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.6462</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -675,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FC Juarez vs Pumas UNAM</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>FC Juarez</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Pumas UNAM</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
+          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19532549</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785417902</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>43.759691</t>
+          <t>6.849301</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
+          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,23 +763,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>21.56505</t>
+          <t>14.25999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -779,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
+          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785417868</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>48.325042</t>
+          <t>19.534233</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
+          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -859,28 +875,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>24.09035</t>
+          <t>47.67</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>Atletico San Luis vs Tijuana</t>
@@ -898,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785410369</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>50.850343</t>
+          <t>138.676364</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
+          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -966,17 +990,17 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14.01714</t>
+          <t>28.2797</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.6462</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -987,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>FC Juarez vs Pumas UNAM</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>FC Juarez</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
+          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532549</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1032,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785410369</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>40.777135</t>
+          <t>43.759691</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
+          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1070,17 +1094,17 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>23.37583</t>
+          <t>21.56505</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1091,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1136,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785409703</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>50.135828</t>
+          <t>48.325042</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
+          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1171,31 +1195,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>24.09035</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1203,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1248,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785409538</t>
+          <t>1785410369</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>120.294479</t>
+          <t>50.850343</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,28 +1291,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
+          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>14.01714</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1307,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
+          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1352,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785369486</t>
+          <t>1785410369</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>41.166667</t>
+          <t>40.777135</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,39 +1395,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
+          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>36.47</t>
+          <t>23.37583</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2737</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1434,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1464,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785356693</t>
+          <t>1785409703</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1474,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>133.223744</t>
+          <t>50.135828</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,12 +1499,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1506,12 +1514,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24.51</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5938</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1521,32 +1529,32 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>CD Guadalajara Chivas</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>CD Guadalajara Chivas</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1576,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785409538</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1586,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>120.294479</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1611,31 +1619,23 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Santos Laguna</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1643,27 +1643,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1688,17 +1688,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785369486</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>41.166667</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,12 +1715,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1730,12 +1730,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>36.47</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.2737</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1755,27 +1755,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1800,17 +1800,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,110 +1827,446 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.5938</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1785345076</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1.684211</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>39.56</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Santos Laguna</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Club America vs Santos Laguna</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Club America</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Santos Laguna</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19546221</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1785287219</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1785711600</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>304.307692</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 16:03:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
+          <t>0x069159bb290d05216d5386f3be0c95aaf362689433b534bce3c2c3cb61245830</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>178.29</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.3413</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,24 +561,24 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Atletico San Luis</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Tijuana</t>
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785418294</t>
+          <t>1785423749</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>445.725</t>
+          <t>5.040293</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
+          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>178.29</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
+          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785417902</t>
+          <t>1785418294</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6.849301</t>
+          <t>445.725</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
+          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14.25999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785417868</t>
+          <t>1785417902</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>19.534233</t>
+          <t>6.849301</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
+          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -882,47 +882,47 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>47.67</t>
+          <t>14.25999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785417868</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>138.676364</t>
+          <t>19.534233</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
+          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -987,15 +987,19 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>28.2797</t>
+          <t>47.67</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.6462</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1003,7 +1007,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1011,27 +1019,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>FC Juarez vs Pumas UNAM</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>FC Juarez</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pumas UNAM</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19532549</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1066,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>43.759691</t>
+          <t>138.676364</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,7 +1091,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
+          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1094,17 +1102,17 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>21.56505</t>
+          <t>28.2797</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.6462</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1115,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>FC Juarez vs Pumas UNAM</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>FC Juarez</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
+          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532549</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1165,12 +1173,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>48.325042</t>
+          <t>43.759691</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
+          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1198,17 +1206,17 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>24.09035</t>
+          <t>21.56505</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1219,27 +1227,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1272,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785410369</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>50.850343</t>
+          <t>48.325042</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
+          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1302,17 +1310,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>14.01714</t>
+          <t>24.09035</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Liga MX</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1338,7 +1346,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1378,7 +1386,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>40.777135</t>
+          <t>50.850343</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1403,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
+          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1406,17 +1414,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>23.37583</t>
+          <t>14.01714</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1442,7 +1450,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1472,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785409703</t>
+          <t>1785410369</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>50.135828</t>
+          <t>40.777135</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
+          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1507,31 +1515,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>23.37583</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1539,27 +1539,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1584,17 +1584,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785409538</t>
+          <t>1785409703</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>120.294479</t>
+          <t>50.135828</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,31 +1611,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
+          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>24.51</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1658,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
+          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1688,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785369486</t>
+          <t>1785409538</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1698,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>41.166667</t>
+          <t>120.294479</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,39 +1723,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
+          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>36.47</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2737</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1755,27 +1755,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1800,17 +1800,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785356693</t>
+          <t>1785369486</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>133.223744</t>
+          <t>41.166667</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,12 +1827,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1842,12 +1842,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>36.47</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5938</t>
+          <t>1.2737</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1867,27 +1867,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1912,17 +1912,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,12 +1939,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1979,27 +1979,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2024,17 +2024,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,12 +2051,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2091,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2136,17 +2136,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,110 +2163,222 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 18:04:32 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x069159bb290d05216d5386f3be0c95aaf362689433b534bce3c2c3cb61245830</t>
+          <t>0x77b65cc254c4e2c182f338e283bf4bfdd20f64a31b22f7c7ffaf4f7fd804a34d</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,47 +546,47 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>10.01972</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3413</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0x02b765bb20cec10921b66af424aab9699fb9c107684131f78fe6911a8be5b095</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785423749</t>
+          <t>1785431683</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>5.040293</t>
+          <t>17.539991</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
+          <t>0x069159bb290d05216d5386f3be0c95aaf362689433b534bce3c2c3cb61245830</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>178.29</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.3413</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,24 +673,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>Atletico San Luis</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Tijuana</t>
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785418294</t>
+          <t>1785423749</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>445.725</t>
+          <t>5.040293</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
+          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +770,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>178.29</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
+          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785417902</t>
+          <t>1785418294</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6.849301</t>
+          <t>445.725</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +867,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
+          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>14.25999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785417868</t>
+          <t>1785417902</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>19.534233</t>
+          <t>6.849301</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
+          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -994,47 +994,47 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>47.67</t>
+          <t>14.25999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785417868</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>138.676364</t>
+          <t>19.534233</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
+          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1099,15 +1099,19 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>28.2797</t>
+          <t>47.67</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6462</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1115,7 +1119,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1123,27 +1131,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>FC Juarez vs Pumas UNAM</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>FC Juarez</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Pumas UNAM</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19532549</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1178,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>43.759691</t>
+          <t>138.676364</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
+          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1206,17 +1214,17 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>21.56505</t>
+          <t>28.2797</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.6462</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1227,27 +1235,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>FC Juarez vs Pumas UNAM</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>FC Juarez</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
+          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532549</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1277,12 +1285,12 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.325042</t>
+          <t>43.759691</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1307,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
+          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1310,17 +1318,17 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>24.09035</t>
+          <t>21.56505</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1331,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785410369</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>50.850343</t>
+          <t>48.325042</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
+          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1414,17 +1422,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14.01714</t>
+          <t>24.09035</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Liga MX</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1450,7 +1458,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1490,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>40.777135</t>
+          <t>50.850343</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1515,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
+          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1518,17 +1526,17 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23.37583</t>
+          <t>14.01714</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1554,7 +1562,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785409703</t>
+          <t>1785410369</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>50.135828</t>
+          <t>40.777135</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
+          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1619,31 +1627,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>23.37583</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1651,27 +1651,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1696,17 +1696,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785409538</t>
+          <t>1785409703</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>120.294479</t>
+          <t>50.135828</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,31 +1723,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
+          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>24.51</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1770,7 +1778,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
+          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1800,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785369486</t>
+          <t>1785409538</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1810,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>41.166667</t>
+          <t>120.294479</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1827,39 +1835,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
+          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>36.47</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2737</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1867,27 +1867,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1912,17 +1912,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785356693</t>
+          <t>1785369486</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>133.223744</t>
+          <t>41.166667</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,12 +1939,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>36.47</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5938</t>
+          <t>1.2737</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1979,27 +1979,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2024,17 +2024,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,12 +2051,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2091,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2136,17 +2136,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,12 +2163,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2203,27 +2203,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,110 +2275,222 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-07-30 23:02:24 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Liga MX/trades.xlsx
+++ b/data/sxbet/ligas/Liga MX/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x67f236378642e650288072537c5ca321fcdb81c90ca456e20e4ebe81a366bdca</t>
+          <t>0x834cc413fad1ae476b3abcc079d6dfdf4999377ba031308e745aedd36635dcc9</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>59.99</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4075</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>FC Juarez vs Pumas UNAM</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>FC Juarez</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
+          <t>0xe673b69f0e7e808a0e8ad5fdd3f1565a51ba11f9cf701037090d8a39c9627c8c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532549</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785441578</t>
+          <t>1785447000</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>147.214724</t>
+          <t>5.038062</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x77b65cc254c4e2c182f338e283bf4bfdd20f64a31b22f7c7ffaf4f7fd804a34d</t>
+          <t>0x67f236378642e650288072537c5ca321fcdb81c90ca456e20e4ebe81a366bdca</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.01972</t>
+          <t>59.99</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5713</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x02b765bb20cec10921b66af424aab9699fb9c107684131f78fe6911a8be5b095</t>
+          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785431683</t>
+          <t>1785441578</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>17.539991</t>
+          <t>147.214724</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x069159bb290d05216d5386f3be0c95aaf362689433b534bce3c2c3cb61245830</t>
+          <t>0x77b65cc254c4e2c182f338e283bf4bfdd20f64a31b22f7c7ffaf4f7fd804a34d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,47 +770,47 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>10.01972</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3413</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0x02b765bb20cec10921b66af424aab9699fb9c107684131f78fe6911a8be5b095</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785423749</t>
+          <t>1785431683</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>5.040293</t>
+          <t>17.539991</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +867,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
+          <t>0x069159bb290d05216d5386f3be0c95aaf362689433b534bce3c2c3cb61245830</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,12 +882,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>178.29</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.3413</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,24 +897,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>Atletico San Luis</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Tijuana</t>
@@ -922,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785418294</t>
+          <t>1785423749</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>445.725</t>
+          <t>5.040293</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,12 +979,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
+          <t>0x71fcd1567bd30dc94507812dc6e17f69a52d84fead2eaeb04523d2743533ccb4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x7CA12ef070eAc708909d595aF0A62fb964e82eB8</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -994,22 +994,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>178.29</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
+          <t>0x1a106c1f8d59c1f1d790c22eb151671bed73890f10324638cf193b5697500ae0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785417902</t>
+          <t>1785418294</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6.849301</t>
+          <t>445.725</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,12 +1091,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
+          <t>0xaeee6d75ef70379c96b94a2f46b5fd4c6503d6a05b2d06a1f7238d76fde35a9d</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>14.25999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785417868</t>
+          <t>1785417902</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>19.534233</t>
+          <t>6.849301</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
+          <t>0x3d642d7df577d36818b87fd5c76ece4139a672a8a992a2d655c002d912658141</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1218,47 +1218,47 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>47.67</t>
+          <t>14.25999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Atletico San Luis vs Tijuana</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Atletico San Luis</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>Tijuana</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Liga MX</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Atletico San Luis vs Tijuana</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Atletico San Luis</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Tijuana</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
+          <t>0xdb0514e2fdc4a5937810ecb6df929a2f75884419f98f2d1904b1111b72e9eb93</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785410371</t>
+          <t>1785417868</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>138.676364</t>
+          <t>19.534233</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
+          <t>0xc3151807b27d29dcfb95836634f5d2e33c9b84ac59f63ecae555b066a1ef4761</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1323,15 +1323,19 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>28.2797</t>
+          <t>47.67</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.6462</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1339,7 +1343,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1347,27 +1355,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>FC Juarez vs Pumas UNAM</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>FC Juarez</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Pumas UNAM</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
+          <t>0x9ad4e5af1e570a88eae866cab4f39eaa270c5f08bc37f41739734fc51d0649cb</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19532549</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1402,7 +1410,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>43.759691</t>
+          <t>138.676364</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,7 +1427,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
+          <t>0xba937b7e81637cccd1e2a5724a8e43ea92d25bcfcbfc8f93217a79a9ff1c92e9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1430,17 +1438,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>21.56505</t>
+          <t>28.2797</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.6462</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1451,27 +1459,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>FC Juarez vs Pumas UNAM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>FC Juarez</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Pumas UNAM</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
+          <t>0x37bc9570caeea6400aa2544b7d0f8b9753fe12bfa6d8d9e78a9d709530ff5427</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532549</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1501,12 +1509,12 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>48.325042</t>
+          <t>43.759691</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,7 +1531,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
+          <t>0x2b451cd534ebb127bdd4f7f8b7f88d5323bad8bcad151a09bc22d4c9d6c3c192</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1534,17 +1542,17 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>24.09035</t>
+          <t>21.56505</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.4737</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (1)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1555,27 +1563,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0x5db77b39e9d7e955a1d762e1dfd9f8b3b172358749461d773ccd7c72d1ec5134</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1600,17 +1608,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785410369</t>
+          <t>1785410371</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>50.850343</t>
+          <t>48.325042</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,7 +1635,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
+          <t>0xd2702fa11ea4b232bb27eb16780ea0c440d8369212c3970419bbdf135ad614fa</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1638,17 +1646,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>14.01714</t>
+          <t>24.09035</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4737</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Liga MX</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1674,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1714,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>40.777135</t>
+          <t>50.850343</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,7 +1739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
+          <t>0xb9659363a3fc03307594f98c5b81f447a54f2f09090d06e4db8c7accd0cf38a1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1742,17 +1750,17 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23.37583</t>
+          <t>14.01714</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.4663</t>
+          <t>1.3438</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Liga MX</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1778,7 +1786,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
+          <t>0xbe85f5ed784cd5f9e4bc5d9113a2dbce8b0ac350d04832099b72c3c6d7818877</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1808,7 +1816,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785409703</t>
+          <t>1785410369</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1826,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>50.135828</t>
+          <t>40.777135</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
+          <t>0x9a110e5fedcb97a1c8c579a685c7635dc84185e4038298c47f2153c6a5c8b954</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1843,31 +1851,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>24.51</t>
+          <t>23.37583</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2037</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Puebla</t>
-        </is>
-      </c>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1875,27 +1875,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
+          <t>0x521d2f3e5e251999c6ac8d43c9e45301b3eb455e632a4e16563909c0d61dddc3</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,17 +1920,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785409538</t>
+          <t>1785409703</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>120.294479</t>
+          <t>50.135828</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,31 +1947,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
+          <t>0x6a48ab839278716d42162ff59711cc25c14bd8a5d3689d134725271792294c31</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>24.51</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.2037</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -1994,7 +2002,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
+          <t>0xfe04744982f35a9716b90547fa285954d58ae53b5ffd645128f4f12d776f1b14</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2024,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785369486</t>
+          <t>1785409538</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>41.166667</t>
+          <t>120.294479</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,39 +2059,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
+          <t>0xfdf455bbc71d71d6827140dbbb2669c1b6a2ee70b65b04ab117f7815d089f1b1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>36.47</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2737</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Liga MX</t>
@@ -2091,27 +2091,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Atletico San Luis vs Tijuana</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Atletico San Luis</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Tijuana</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
+          <t>0xc0c95c54c55f4bf1cae851478372b5223674ce25544abc71bd8eb115bf09be02</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19532655</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2136,17 +2136,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785356693</t>
+          <t>1785369486</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1785553200</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>133.223744</t>
+          <t>41.166667</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,12 +2163,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
+          <t>0xf3a74abf2844e6928d04caa7acb52d3ca95905545b7fb4674fde8fa057a5c3e0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xf068eF8DF8f47185D02d59Bb33d9eC7A057a571E</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>36.47</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5938</t>
+          <t>1.2737</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2203,27 +2203,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Atletico San Luis vs Tijuana</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Atletico San Luis</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Tijuana</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0xc80816e0843fb9db57cea8c04416c33e871cdc6d3bcbb6807c3703e7043ccdfd</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19532655</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785345076</t>
+          <t>1785356693</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785553200</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.684211</t>
+          <t>133.223744</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
+          <t>0x3b4a78d70e21af26b94ff0c78303a9bb935c0e1ee16c1d51b277692cb3ab0556</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2290,12 +2290,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>39.56</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.5938</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2315,27 +2315,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Club America vs Santos Laguna</t>
+          <t>Puebla vs CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Club America</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Santos Laguna</t>
+          <t>CD Guadalajara Chivas</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19546221</t>
+          <t>L19532532</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2360,17 +2360,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785287219</t>
+          <t>1785345076</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1785711600</t>
+          <t>1785546000</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>304.307692</t>
+          <t>1.684211</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,12 +2387,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+          <t>0x3df8792686cb34cf26d9f4e518a0d3bb8e57fc9537a6c86e827509a1cc6e7a9f</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2402,12 +2402,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.49576</t>
+          <t>39.56</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2427,27 +2427,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Puebla vs CD Guadalajara Chivas</t>
+          <t>Club America vs Santos Laguna</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Puebla</t>
+          <t>Club America</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>CD Guadalajara Chivas</t>
+          <t>Santos Laguna</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+          <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19532532</t>
+          <t>L19546221</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2472,17 +2472,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785283352</t>
+          <t>1785287219</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1785546000</t>
+          <t>1785711600</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>4.185761</t>
+          <t>304.307692</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,110 +2499,222 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>0x8adbc0f011afd6dfa01a9772f962e071de78ad81c7591f1f6ff4ac9bf18d9a18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2.49576</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.5962</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Liga MX</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Puebla vs CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>CD Guadalajara Chivas</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0xcb46a51d354f77fd5bd1744c0c25aa45809a12185fe4e346c524e7ce717970d9</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19532532</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1785283352</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1785546000</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>4.185761</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>0x261e9433f550930dd9a03f754567105ce29e1b0b89b0ebce197de7d54da15f0e</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>9.84849</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>1.13</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Liga MX</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Club America vs Santos Laguna</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Club America</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Santos Laguna</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>0x813e1b7279d5234eab211c2255aaad74d3304de611059f5fb7dae0edbd255db0</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>L19546221</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>1785277583</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>1785711600</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>75.757615</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>